<commit_message>
correccion de ciertas vulnerabilidades he instalacion de googleapis
</commit_message>
<xml_diff>
--- a/datos/excel/6a06af219064f0305ee69cd2/2026-05.xlsx
+++ b/datos/excel/6a06af219064f0305ee69cd2/2026-05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>Día</t>
   </si>
@@ -53,6 +53,15 @@
   </si>
   <si>
     <t>uuuuu</t>
+  </si>
+  <si>
+    <t>martes, 05 de mayo de 2026</t>
+  </si>
+  <si>
+    <t>nichole</t>
+  </si>
+  <si>
+    <t>tukiii</t>
   </si>
   <si>
     <t>viernes, 15 de mayo de 2026</t>
@@ -453,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -534,7 +543,7 @@
     </row>
     <row r="6" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>14</v>
@@ -544,6 +553,20 @@
       </c>
       <c r="D6" s="2" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>15</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correccion de botones he implementacion excel enlazado en tiempo real
</commit_message>
<xml_diff>
--- a/datos/excel/6a06af219064f0305ee69cd2/2026-05.xlsx
+++ b/datos/excel/6a06af219064f0305ee69cd2/2026-05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Día</t>
   </si>
@@ -62,6 +62,12 @@
   </si>
   <si>
     <t>tukiii</t>
+  </si>
+  <si>
+    <t>miércoles, 06 de mayo de 2026</t>
+  </si>
+  <si>
+    <t>hhh</t>
   </si>
   <si>
     <t>viernes, 15 de mayo de 2026</t>
@@ -462,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -557,7 +563,7 @@
     </row>
     <row r="7" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>17</v>
@@ -566,7 +572,21 @@
         <v>18</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>19</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>